<commit_message>
Test The Sales Report Data
</commit_message>
<xml_diff>
--- a/Excel/Sales-Report.xlsx
+++ b/Excel/Sales-Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\j-l-data-science-data-analytics\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Tests\j-l-data-science-data-analytics\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B33EE9F-60DE-44E3-AD66-163A99005047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A808917-FA0E-44BE-9B35-263FC5F3E98A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="4" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="11" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -327,7 +327,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -343,6 +343,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="45">
@@ -394,9 +397,6 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -420,6 +420,9 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -503,8 +506,7 @@
           </a:sp3d>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="5"/>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -548,6 +550,82 @@
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
           </c:extLst>
         </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+          <a:sp3d contourW="25400">
+            <a:contourClr>
+              <a:schemeClr val="lt1"/>
+            </a:contourClr>
+          </a:sp3d>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+          <a:sp3d contourW="25400">
+            <a:contourClr>
+              <a:schemeClr val="lt1"/>
+            </a:contourClr>
+          </a:sp3d>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+          <a:sp3d contourW="25400">
+            <a:contourClr>
+              <a:schemeClr val="lt1"/>
+            </a:contourClr>
+          </a:sp3d>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+          <a:sp3d contourW="25400">
+            <a:contourClr>
+              <a:schemeClr val="lt1"/>
+            </a:contourClr>
+          </a:sp3d>
+        </c:spPr>
       </c:pivotFmt>
     </c:pivotFmts>
     <c:view3D>
@@ -626,6 +704,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-D9AF-43EB-A4A4-AC78705249B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -646,6 +729,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-D9AF-43EB-A4A4-AC78705249B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -666,6 +754,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-D9AF-43EB-A4A4-AC78705249B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -686,6 +779,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-D9AF-43EB-A4A4-AC78705249B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -3782,7 +3880,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{268A8983-0403-4910-98F7-0770A3DB0E11}" name="PivotTable3" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{268A8983-0403-4910-98F7-0770A3DB0E11}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -3832,16 +3930,64 @@
     <dataField name="Sum of Sale Price" fld="5" baseField="0" baseItem="0" numFmtId="44"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="0">
+    <format dxfId="1">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
-  <chartFormats count="1">
+  <chartFormats count="5">
     <chartFormat chart="2" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
@@ -3860,7 +4006,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{90D4FB98-9A71-4127-A66B-463DBC99FC24}" name="Table1" displayName="Table1" ref="A1:K1048576" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{90D4FB98-9A71-4127-A66B-463DBC99FC24}" name="Table1" displayName="Table1" ref="A1:K1048576" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:K1048576" xr:uid="{90D4FB98-9A71-4127-A66B-463DBC99FC24}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K177">
     <sortCondition ref="B2:B177"/>
   </sortState>
@@ -4204,10 +4351,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98733610-7D45-4653-9B5E-324F90078C3D}">
   <dimension ref="A3:B8"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:2">
@@ -4267,21 +4414,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K176"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="13.75" customWidth="1"/>
-    <col min="2" max="2" width="20.25" customWidth="1"/>
-    <col min="3" max="3" width="14.375" customWidth="1"/>
-    <col min="4" max="4" width="19.875" customWidth="1"/>
+    <col min="1" max="1" width="13.69921875" customWidth="1"/>
+    <col min="2" max="2" width="20.19921875" customWidth="1"/>
+    <col min="3" max="3" width="14.3984375" customWidth="1"/>
+    <col min="4" max="4" width="19.8984375" customWidth="1"/>
     <col min="5" max="5" width="11.5" customWidth="1"/>
-    <col min="6" max="6" width="14.25" customWidth="1"/>
-    <col min="8" max="8" width="23.125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.75" customWidth="1"/>
-    <col min="11" max="11" width="14.125" customWidth="1"/>
+    <col min="6" max="6" width="14.19921875" customWidth="1"/>
+    <col min="8" max="8" width="23.09765625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="13.69921875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.69921875" customWidth="1"/>
+    <col min="11" max="11" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="47.25">
+    <row r="1" spans="1:11" ht="46.8">
       <c r="A1" s="4" t="s">
         <v>22</v>
       </c>
@@ -4336,11 +4483,11 @@
         <v>98.4</v>
       </c>
       <c r="G2" s="5">
-        <f>F2-E2</f>
+        <f t="shared" ref="G2:G33" si="0">F2-E2</f>
         <v>40.100000000000009</v>
       </c>
       <c r="H2" s="3">
-        <f>IF(F2&gt;50, G2*0.2, G2*0.1)</f>
+        <f t="shared" ref="H2:H33" si="1">IF(F2&gt;50, G2*0.2, G2*0.1)</f>
         <v>8.0200000000000014</v>
       </c>
       <c r="I2" t="s">
@@ -4373,11 +4520,11 @@
         <v>16.3</v>
       </c>
       <c r="G3" s="5">
-        <f>F3-E3</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H3" s="7">
-        <f>IF(F3&gt;50, G3*0.2, G3*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I3" t="s">
@@ -4410,11 +4557,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G4" s="5">
-        <f>F4-E4</f>
+        <f t="shared" si="0"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H4" s="3">
-        <f>IF(F4&gt;50, G4*0.2, G4*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I4" t="s">
@@ -4447,11 +4594,11 @@
         <v>502</v>
       </c>
       <c r="G5" s="5">
-        <f>F5-E5</f>
+        <f t="shared" si="0"/>
         <v>158</v>
       </c>
       <c r="H5" s="3">
-        <f>IF(F5&gt;50, G5*0.2, G5*0.1)</f>
+        <f t="shared" si="1"/>
         <v>31.6</v>
       </c>
       <c r="I5" t="s">
@@ -4484,11 +4631,11 @@
         <v>8</v>
       </c>
       <c r="G6" s="5">
-        <f>F6-E6</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H6" s="3">
-        <f>IF(F6&gt;50, G6*0.2, G6*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I6" t="s">
@@ -4521,11 +4668,11 @@
         <v>98.4</v>
       </c>
       <c r="G7" s="5">
-        <f>F7-E7</f>
+        <f t="shared" si="0"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H7" s="3">
-        <f>IF(F7&gt;50, G7*0.2, G7*0.1)</f>
+        <f t="shared" si="1"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I7" t="s">
@@ -4558,11 +4705,11 @@
         <v>8</v>
       </c>
       <c r="G8" s="5">
-        <f>F8-E8</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H8" s="3">
-        <f>IF(F8&gt;50, G8*0.2, G8*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I8" t="s">
@@ -4595,11 +4742,11 @@
         <v>16.3</v>
       </c>
       <c r="G9" s="5">
-        <f>F9-E9</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H9" s="3">
-        <f>IF(F9&gt;50, G9*0.2, G9*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I9" t="s">
@@ -4632,11 +4779,11 @@
         <v>8</v>
       </c>
       <c r="G10" s="5">
-        <f>F10-E10</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H10" s="3">
-        <f>IF(F10&gt;50, G10*0.2, G10*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I10" t="s">
@@ -4669,11 +4816,11 @@
         <v>16.3</v>
       </c>
       <c r="G11" s="5">
-        <f>F11-E11</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H11" s="3">
-        <f>IF(F11&gt;50, G11*0.2, G11*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I11" t="s">
@@ -4706,11 +4853,11 @@
         <v>16.3</v>
       </c>
       <c r="G12" s="5">
-        <f>F12-E12</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H12" s="3">
-        <f>IF(F12&gt;50, G12*0.2, G12*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I12" t="s">
@@ -4743,11 +4890,11 @@
         <v>87</v>
       </c>
       <c r="G13" s="5">
-        <f>F13-E13</f>
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="H13" s="3">
-        <f>IF(F13&gt;50, G13*0.2, G13*0.1)</f>
+        <f t="shared" si="1"/>
         <v>8.4</v>
       </c>
       <c r="I13" t="s">
@@ -4780,11 +4927,11 @@
         <v>7</v>
       </c>
       <c r="G14" s="5">
-        <f>F14-E14</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H14" s="3">
-        <f>IF(F14&gt;50, G14*0.2, G14*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I14" t="s">
@@ -4817,11 +4964,11 @@
         <v>502</v>
       </c>
       <c r="G15" s="5">
-        <f>F15-E15</f>
+        <f t="shared" si="0"/>
         <v>158</v>
       </c>
       <c r="H15" s="3">
-        <f>IF(F15&gt;50, G15*0.2, G15*0.1)</f>
+        <f t="shared" si="1"/>
         <v>31.6</v>
       </c>
       <c r="I15" t="s">
@@ -4854,11 +5001,11 @@
         <v>16.3</v>
       </c>
       <c r="G16" s="5">
-        <f>F16-E16</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H16" s="3">
-        <f>IF(F16&gt;50, G16*0.2, G16*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I16" t="s">
@@ -4891,11 +5038,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G17" s="5">
-        <f>F17-E17</f>
+        <f t="shared" si="0"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H17" s="3">
-        <f>IF(F17&gt;50, G17*0.2, G17*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I17" t="s">
@@ -4928,11 +5075,11 @@
         <v>124</v>
       </c>
       <c r="G18" s="5">
-        <f>F18-E18</f>
+        <f t="shared" si="0"/>
         <v>64</v>
       </c>
       <c r="H18" s="3">
-        <f>IF(F18&gt;50, G18*0.2, G18*0.1)</f>
+        <f t="shared" si="1"/>
         <v>12.8</v>
       </c>
       <c r="I18" t="s">
@@ -4965,11 +5112,11 @@
         <v>8</v>
       </c>
       <c r="G19" s="5">
-        <f>F19-E19</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H19" s="3">
-        <f>IF(F19&gt;50, G19*0.2, G19*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I19" t="s">
@@ -5002,11 +5149,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G20" s="5">
-        <f>F20-E20</f>
+        <f t="shared" si="0"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H20" s="3">
-        <f>IF(F20&gt;50, G20*0.2, G20*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I20" t="s">
@@ -5039,11 +5186,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G21" s="5">
-        <f>F21-E21</f>
+        <f t="shared" si="0"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H21" s="3">
-        <f>IF(F21&gt;50, G21*0.2, G21*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I21" t="s">
@@ -5076,11 +5223,11 @@
         <v>8</v>
       </c>
       <c r="G22" s="5">
-        <f>F22-E22</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H22" s="3">
-        <f>IF(F22&gt;50, G22*0.2, G22*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I22" t="s">
@@ -5113,11 +5260,11 @@
         <v>16.3</v>
       </c>
       <c r="G23" s="5">
-        <f>F23-E23</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H23" s="3">
-        <f>IF(F23&gt;50, G23*0.2, G23*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I23" t="s">
@@ -5150,11 +5297,11 @@
         <v>8</v>
       </c>
       <c r="G24" s="5">
-        <f>F24-E24</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H24" s="3">
-        <f>IF(F24&gt;50, G24*0.2, G24*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I24" t="s">
@@ -5187,11 +5334,11 @@
         <v>7</v>
       </c>
       <c r="G25" s="5">
-        <f>F25-E25</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H25" s="3">
-        <f>IF(F25&gt;50, G25*0.2, G25*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I25" t="s">
@@ -5224,11 +5371,11 @@
         <v>16.3</v>
       </c>
       <c r="G26" s="5">
-        <f>F26-E26</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H26" s="3">
-        <f>IF(F26&gt;50, G26*0.2, G26*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I26" t="s">
@@ -5261,11 +5408,11 @@
         <v>14</v>
       </c>
       <c r="G27" s="5">
-        <f>F27-E27</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H27" s="3">
-        <f>IF(F27&gt;50, G27*0.2, G27*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I27" t="s">
@@ -5298,11 +5445,11 @@
         <v>14</v>
       </c>
       <c r="G28" s="5">
-        <f>F28-E28</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H28" s="3">
-        <f>IF(F28&gt;50, G28*0.2, G28*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I28" t="s">
@@ -5335,11 +5482,11 @@
         <v>502</v>
       </c>
       <c r="G29" s="5">
-        <f>F29-E29</f>
+        <f t="shared" si="0"/>
         <v>158</v>
       </c>
       <c r="H29" s="3">
-        <f>IF(F29&gt;50, G29*0.2, G29*0.1)</f>
+        <f t="shared" si="1"/>
         <v>31.6</v>
       </c>
       <c r="I29" t="s">
@@ -5372,11 +5519,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G30" s="5">
-        <f>F30-E30</f>
+        <f t="shared" si="0"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H30" s="3">
-        <f>IF(F30&gt;50, G30*0.2, G30*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I30" t="s">
@@ -5409,11 +5556,11 @@
         <v>87</v>
       </c>
       <c r="G31" s="5">
-        <f>F31-E31</f>
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="H31" s="3">
-        <f>IF(F31&gt;50, G31*0.2, G31*0.1)</f>
+        <f t="shared" si="1"/>
         <v>8.4</v>
       </c>
       <c r="I31" t="s">
@@ -5446,11 +5593,11 @@
         <v>8</v>
       </c>
       <c r="G32" s="5">
-        <f>F32-E32</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H32" s="3">
-        <f>IF(F32&gt;50, G32*0.2, G32*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
       <c r="I32" t="s">
@@ -5483,11 +5630,11 @@
         <v>16.3</v>
       </c>
       <c r="G33" s="5">
-        <f>F33-E33</f>
+        <f t="shared" si="0"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H33" s="3">
-        <f>IF(F33&gt;50, G33*0.2, G33*0.1)</f>
+        <f t="shared" si="1"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I33" t="s">
@@ -5520,11 +5667,11 @@
         <v>98.4</v>
       </c>
       <c r="G34" s="5">
-        <f>F34-E34</f>
+        <f t="shared" ref="G34:G65" si="2">F34-E34</f>
         <v>40.100000000000009</v>
       </c>
       <c r="H34" s="3">
-        <f>IF(F34&gt;50, G34*0.2, G34*0.1)</f>
+        <f t="shared" ref="H34:H65" si="3">IF(F34&gt;50, G34*0.2, G34*0.1)</f>
         <v>8.0200000000000014</v>
       </c>
       <c r="I34" t="s">
@@ -5557,11 +5704,11 @@
         <v>16.3</v>
       </c>
       <c r="G35" s="5">
-        <f>F35-E35</f>
+        <f t="shared" si="2"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H35" s="3">
-        <f>IF(F35&gt;50, G35*0.2, G35*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I35" t="s">
@@ -5594,11 +5741,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G36" s="5">
-        <f>F36-E36</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H36" s="3">
-        <f>IF(F36&gt;50, G36*0.2, G36*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I36" t="s">
@@ -5631,11 +5778,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G37" s="5">
-        <f>F37-E37</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H37" s="3">
-        <f>IF(F37&gt;50, G37*0.2, G37*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I37" t="s">
@@ -5668,11 +5815,11 @@
         <v>77</v>
       </c>
       <c r="G38" s="5">
-        <f>F38-E38</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="H38" s="3">
-        <f>IF(F38&gt;50, G38*0.2, G38*0.1)</f>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="I38" t="s">
@@ -5705,11 +5852,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G39" s="5">
-        <f>F39-E39</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H39" s="3">
-        <f>IF(F39&gt;50, G39*0.2, G39*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I39" t="s">
@@ -5742,11 +5889,11 @@
         <v>16.3</v>
       </c>
       <c r="G40" s="5">
-        <f>F40-E40</f>
+        <f t="shared" si="2"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H40" s="3">
-        <f>IF(F40&gt;50, G40*0.2, G40*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I40" t="s">
@@ -5779,11 +5926,11 @@
         <v>8</v>
       </c>
       <c r="G41" s="5">
-        <f>F41-E41</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H41" s="3">
-        <f>IF(F41&gt;50, G41*0.2, G41*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I41" t="s">
@@ -5816,11 +5963,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G42" s="5">
-        <f>F42-E42</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H42" s="3">
-        <f>IF(F42&gt;50, G42*0.2, G42*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I42" t="s">
@@ -5853,11 +6000,11 @@
         <v>502</v>
       </c>
       <c r="G43" s="5">
-        <f>F43-E43</f>
+        <f t="shared" si="2"/>
         <v>158</v>
       </c>
       <c r="H43" s="3">
-        <f>IF(F43&gt;50, G43*0.2, G43*0.1)</f>
+        <f t="shared" si="3"/>
         <v>31.6</v>
       </c>
       <c r="I43" t="s">
@@ -5890,11 +6037,11 @@
         <v>124</v>
       </c>
       <c r="G44" s="5">
-        <f>F44-E44</f>
+        <f t="shared" si="2"/>
         <v>64</v>
       </c>
       <c r="H44" s="3">
-        <f>IF(F44&gt;50, G44*0.2, G44*0.1)</f>
+        <f t="shared" si="3"/>
         <v>12.8</v>
       </c>
       <c r="I44" t="s">
@@ -5927,11 +6074,11 @@
         <v>16.3</v>
       </c>
       <c r="G45" s="5">
-        <f>F45-E45</f>
+        <f t="shared" si="2"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H45" s="3">
-        <f>IF(F45&gt;50, G45*0.2, G45*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I45" t="s">
@@ -5964,11 +6111,11 @@
         <v>502</v>
       </c>
       <c r="G46" s="5">
-        <f>F46-E46</f>
+        <f t="shared" si="2"/>
         <v>158</v>
       </c>
       <c r="H46" s="3">
-        <f>IF(F46&gt;50, G46*0.2, G46*0.1)</f>
+        <f t="shared" si="3"/>
         <v>31.6</v>
       </c>
       <c r="I46" t="s">
@@ -6001,11 +6148,11 @@
         <v>14</v>
       </c>
       <c r="G47" s="5">
-        <f>F47-E47</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H47" s="3">
-        <f>IF(F47&gt;50, G47*0.2, G47*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I47" t="s">
@@ -6038,11 +6185,11 @@
         <v>77</v>
       </c>
       <c r="G48" s="5">
-        <f>F48-E48</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="H48" s="3">
-        <f>IF(F48&gt;50, G48*0.2, G48*0.1)</f>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="I48" t="s">
@@ -6075,11 +6222,11 @@
         <v>502</v>
       </c>
       <c r="G49" s="5">
-        <f>F49-E49</f>
+        <f t="shared" si="2"/>
         <v>158</v>
       </c>
       <c r="H49" s="3">
-        <f>IF(F49&gt;50, G49*0.2, G49*0.1)</f>
+        <f t="shared" si="3"/>
         <v>31.6</v>
       </c>
       <c r="I49" t="s">
@@ -6112,11 +6259,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G50" s="5">
-        <f>F50-E50</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H50" s="3">
-        <f>IF(F50&gt;50, G50*0.2, G50*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I50" t="s">
@@ -6149,11 +6296,11 @@
         <v>16.3</v>
       </c>
       <c r="G51" s="5">
-        <f>F51-E51</f>
+        <f t="shared" si="2"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H51" s="3">
-        <f>IF(F51&gt;50, G51*0.2, G51*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I51" t="s">
@@ -6186,11 +6333,11 @@
         <v>14</v>
       </c>
       <c r="G52" s="5">
-        <f>F52-E52</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H52" s="3">
-        <f>IF(F52&gt;50, G52*0.2, G52*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I52" t="s">
@@ -6223,11 +6370,11 @@
         <v>77</v>
       </c>
       <c r="G53" s="5">
-        <f>F53-E53</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="H53" s="3">
-        <f>IF(F53&gt;50, G53*0.2, G53*0.1)</f>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="I53" t="s">
@@ -6260,11 +6407,11 @@
         <v>124</v>
       </c>
       <c r="G54" s="5">
-        <f>F54-E54</f>
+        <f t="shared" si="2"/>
         <v>64</v>
       </c>
       <c r="H54" s="3">
-        <f>IF(F54&gt;50, G54*0.2, G54*0.1)</f>
+        <f t="shared" si="3"/>
         <v>12.8</v>
       </c>
       <c r="I54" t="s">
@@ -6297,11 +6444,11 @@
         <v>87</v>
       </c>
       <c r="G55" s="5">
-        <f>F55-E55</f>
+        <f t="shared" si="2"/>
         <v>42</v>
       </c>
       <c r="H55" s="3">
-        <f>IF(F55&gt;50, G55*0.2, G55*0.1)</f>
+        <f t="shared" si="3"/>
         <v>8.4</v>
       </c>
       <c r="I55" t="s">
@@ -6334,11 +6481,11 @@
         <v>14</v>
       </c>
       <c r="G56" s="5">
-        <f>F56-E56</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H56" s="3">
-        <f>IF(F56&gt;50, G56*0.2, G56*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I56" t="s">
@@ -6371,11 +6518,11 @@
         <v>8</v>
       </c>
       <c r="G57" s="5">
-        <f>F57-E57</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H57" s="3">
-        <f>IF(F57&gt;50, G57*0.2, G57*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I57" t="s">
@@ -6408,11 +6555,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G58" s="5">
-        <f>F58-E58</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H58" s="3">
-        <f>IF(F58&gt;50, G58*0.2, G58*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I58" t="s">
@@ -6445,11 +6592,11 @@
         <v>14</v>
       </c>
       <c r="G59" s="5">
-        <f>F59-E59</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H59" s="3">
-        <f>IF(F59&gt;50, G59*0.2, G59*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I59" t="s">
@@ -6482,11 +6629,11 @@
         <v>124</v>
       </c>
       <c r="G60" s="5">
-        <f>F60-E60</f>
+        <f t="shared" si="2"/>
         <v>64</v>
       </c>
       <c r="H60" s="3">
-        <f>IF(F60&gt;50, G60*0.2, G60*0.1)</f>
+        <f t="shared" si="3"/>
         <v>12.8</v>
       </c>
       <c r="I60" t="s">
@@ -6519,11 +6666,11 @@
         <v>14</v>
       </c>
       <c r="G61" s="5">
-        <f>F61-E61</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H61" s="3">
-        <f>IF(F61&gt;50, G61*0.2, G61*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I61" t="s">
@@ -6556,11 +6703,11 @@
         <v>8</v>
       </c>
       <c r="G62" s="5">
-        <f>F62-E62</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H62" s="3">
-        <f>IF(F62&gt;50, G62*0.2, G62*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I62" t="s">
@@ -6593,11 +6740,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G63" s="5">
-        <f>F63-E63</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H63" s="3">
-        <f>IF(F63&gt;50, G63*0.2, G63*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I63" t="s">
@@ -6630,11 +6777,11 @@
         <v>8</v>
       </c>
       <c r="G64" s="5">
-        <f>F64-E64</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="H64" s="3">
-        <f>IF(F64&gt;50, G64*0.2, G64*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="I64" t="s">
@@ -6667,11 +6814,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G65" s="5">
-        <f>F65-E65</f>
+        <f t="shared" si="2"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H65" s="3">
-        <f>IF(F65&gt;50, G65*0.2, G65*0.1)</f>
+        <f t="shared" si="3"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I65" t="s">
@@ -6704,11 +6851,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G66" s="5">
-        <f>F66-E66</f>
+        <f t="shared" ref="G66:G97" si="4">F66-E66</f>
         <v>2.9999999999999991</v>
       </c>
       <c r="H66" s="3">
-        <f>IF(F66&gt;50, G66*0.2, G66*0.1)</f>
+        <f t="shared" ref="H66:H97" si="5">IF(F66&gt;50, G66*0.2, G66*0.1)</f>
         <v>0.29999999999999993</v>
       </c>
       <c r="I66" t="s">
@@ -6741,11 +6888,11 @@
         <v>16.3</v>
       </c>
       <c r="G67" s="5">
-        <f>F67-E67</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H67" s="3">
-        <f>IF(F67&gt;50, G67*0.2, G67*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I67" t="s">
@@ -6778,11 +6925,11 @@
         <v>16.3</v>
       </c>
       <c r="G68" s="5">
-        <f>F68-E68</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H68" s="3">
-        <f>IF(F68&gt;50, G68*0.2, G68*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I68" t="s">
@@ -6815,11 +6962,11 @@
         <v>14</v>
       </c>
       <c r="G69" s="5">
-        <f>F69-E69</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H69" s="3">
-        <f>IF(F69&gt;50, G69*0.2, G69*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I69" t="s">
@@ -6852,11 +6999,11 @@
         <v>8</v>
       </c>
       <c r="G70" s="5">
-        <f>F70-E70</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H70" s="3">
-        <f>IF(F70&gt;50, G70*0.2, G70*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I70" t="s">
@@ -6889,11 +7036,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G71" s="5">
-        <f>F71-E71</f>
+        <f t="shared" si="4"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H71" s="3">
-        <f>IF(F71&gt;50, G71*0.2, G71*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I71" t="s">
@@ -6926,11 +7073,11 @@
         <v>8</v>
       </c>
       <c r="G72" s="5">
-        <f>F72-E72</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H72" s="3">
-        <f>IF(F72&gt;50, G72*0.2, G72*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I72" t="s">
@@ -6963,11 +7110,11 @@
         <v>8</v>
       </c>
       <c r="G73" s="5">
-        <f>F73-E73</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H73" s="3">
-        <f>IF(F73&gt;50, G73*0.2, G73*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I73" t="s">
@@ -7000,11 +7147,11 @@
         <v>77</v>
       </c>
       <c r="G74" s="5">
-        <f>F74-E74</f>
+        <f t="shared" si="4"/>
         <v>35</v>
       </c>
       <c r="H74" s="3">
-        <f>IF(F74&gt;50, G74*0.2, G74*0.1)</f>
+        <f t="shared" si="5"/>
         <v>7</v>
       </c>
       <c r="I74" t="s">
@@ -7037,11 +7184,11 @@
         <v>16.3</v>
       </c>
       <c r="G75" s="5">
-        <f>F75-E75</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H75" s="3">
-        <f>IF(F75&gt;50, G75*0.2, G75*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I75" t="s">
@@ -7074,11 +7221,11 @@
         <v>8</v>
       </c>
       <c r="G76" s="5">
-        <f>F76-E76</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H76" s="3">
-        <f>IF(F76&gt;50, G76*0.2, G76*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I76" t="s">
@@ -7111,11 +7258,11 @@
         <v>8</v>
       </c>
       <c r="G77" s="5">
-        <f>F77-E77</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H77" s="3">
-        <f>IF(F77&gt;50, G77*0.2, G77*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I77" t="s">
@@ -7148,11 +7295,11 @@
         <v>98.4</v>
       </c>
       <c r="G78" s="5">
-        <f>F78-E78</f>
+        <f t="shared" si="4"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H78" s="3">
-        <f>IF(F78&gt;50, G78*0.2, G78*0.1)</f>
+        <f t="shared" si="5"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I78" t="s">
@@ -7185,11 +7332,11 @@
         <v>16.3</v>
       </c>
       <c r="G79" s="5">
-        <f>F79-E79</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H79" s="3">
-        <f>IF(F79&gt;50, G79*0.2, G79*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I79" t="s">
@@ -7222,11 +7369,11 @@
         <v>16.3</v>
       </c>
       <c r="G80" s="5">
-        <f>F80-E80</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H80" s="3">
-        <f>IF(F80&gt;50, G80*0.2, G80*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I80" t="s">
@@ -7259,11 +7406,11 @@
         <v>87</v>
       </c>
       <c r="G81" s="5">
-        <f>F81-E81</f>
+        <f t="shared" si="4"/>
         <v>42</v>
       </c>
       <c r="H81" s="3">
-        <f>IF(F81&gt;50, G81*0.2, G81*0.1)</f>
+        <f t="shared" si="5"/>
         <v>8.4</v>
       </c>
       <c r="I81" t="s">
@@ -7296,11 +7443,11 @@
         <v>14</v>
       </c>
       <c r="G82" s="5">
-        <f>F82-E82</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H82" s="3">
-        <f>IF(F82&gt;50, G82*0.2, G82*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I82" t="s">
@@ -7333,11 +7480,11 @@
         <v>8</v>
       </c>
       <c r="G83" s="5">
-        <f>F83-E83</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H83" s="3">
-        <f>IF(F83&gt;50, G83*0.2, G83*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I83" t="s">
@@ -7370,11 +7517,11 @@
         <v>8</v>
       </c>
       <c r="G84" s="5">
-        <f>F84-E84</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H84" s="3">
-        <f>IF(F84&gt;50, G84*0.2, G84*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I84" t="s">
@@ -7407,11 +7554,11 @@
         <v>14</v>
       </c>
       <c r="G85" s="5">
-        <f>F85-E85</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H85" s="3">
-        <f>IF(F85&gt;50, G85*0.2, G85*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I85" t="s">
@@ -7444,11 +7591,11 @@
         <v>98.4</v>
       </c>
       <c r="G86" s="5">
-        <f>F86-E86</f>
+        <f t="shared" si="4"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H86" s="3">
-        <f>IF(F86&gt;50, G86*0.2, G86*0.1)</f>
+        <f t="shared" si="5"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I86" t="s">
@@ -7481,11 +7628,11 @@
         <v>8</v>
       </c>
       <c r="G87" s="5">
-        <f>F87-E87</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H87" s="3">
-        <f>IF(F87&gt;50, G87*0.2, G87*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I87" t="s">
@@ -7518,11 +7665,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G88" s="5">
-        <f>F88-E88</f>
+        <f t="shared" si="4"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H88" s="3">
-        <f>IF(F88&gt;50, G88*0.2, G88*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I88" t="s">
@@ -7555,11 +7702,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G89" s="5">
-        <f>F89-E89</f>
+        <f t="shared" si="4"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H89" s="3">
-        <f>IF(F89&gt;50, G89*0.2, G89*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I89" t="s">
@@ -7592,11 +7739,11 @@
         <v>14</v>
       </c>
       <c r="G90" s="5">
-        <f>F90-E90</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H90" s="3">
-        <f>IF(F90&gt;50, G90*0.2, G90*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I90" t="s">
@@ -7629,11 +7776,11 @@
         <v>16.3</v>
       </c>
       <c r="G91" s="5">
-        <f>F91-E91</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H91" s="3">
-        <f>IF(F91&gt;50, G91*0.2, G91*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I91" t="s">
@@ -7666,11 +7813,11 @@
         <v>16.3</v>
       </c>
       <c r="G92" s="5">
-        <f>F92-E92</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H92" s="3">
-        <f>IF(F92&gt;50, G92*0.2, G92*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I92" t="s">
@@ -7703,11 +7850,11 @@
         <v>16.3</v>
       </c>
       <c r="G93" s="5">
-        <f>F93-E93</f>
+        <f t="shared" si="4"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H93" s="3">
-        <f>IF(F93&gt;50, G93*0.2, G93*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I93" t="s">
@@ -7740,11 +7887,11 @@
         <v>14</v>
       </c>
       <c r="G94" s="5">
-        <f>F94-E94</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H94" s="3">
-        <f>IF(F94&gt;50, G94*0.2, G94*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I94" t="s">
@@ -7777,11 +7924,11 @@
         <v>14</v>
       </c>
       <c r="G95" s="5">
-        <f>F95-E95</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H95" s="3">
-        <f>IF(F95&gt;50, G95*0.2, G95*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I95" t="s">
@@ -7814,11 +7961,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G96" s="5">
-        <f>F96-E96</f>
+        <f t="shared" si="4"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H96" s="3">
-        <f>IF(F96&gt;50, G96*0.2, G96*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I96" t="s">
@@ -7851,11 +7998,11 @@
         <v>14</v>
       </c>
       <c r="G97" s="5">
-        <f>F97-E97</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="H97" s="3">
-        <f>IF(F97&gt;50, G97*0.2, G97*0.1)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="I97" t="s">
@@ -7888,11 +8035,11 @@
         <v>7</v>
       </c>
       <c r="G98" s="5">
-        <f>F98-E98</f>
+        <f t="shared" ref="G98:G129" si="6">F98-E98</f>
         <v>3</v>
       </c>
       <c r="H98" s="3">
-        <f>IF(F98&gt;50, G98*0.2, G98*0.1)</f>
+        <f t="shared" ref="H98:H129" si="7">IF(F98&gt;50, G98*0.2, G98*0.1)</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="I98" t="s">
@@ -7925,11 +8072,11 @@
         <v>16.3</v>
       </c>
       <c r="G99" s="5">
-        <f>F99-E99</f>
+        <f t="shared" si="6"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H99" s="3">
-        <f>IF(F99&gt;50, G99*0.2, G99*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I99" t="s">
@@ -7962,11 +8109,11 @@
         <v>16.3</v>
       </c>
       <c r="G100" s="5">
-        <f>F100-E100</f>
+        <f t="shared" si="6"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H100" s="3">
-        <f>IF(F100&gt;50, G100*0.2, G100*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I100" t="s">
@@ -7999,11 +8146,11 @@
         <v>14</v>
       </c>
       <c r="G101" s="5">
-        <f>F101-E101</f>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="H101" s="3">
-        <f>IF(F101&gt;50, G101*0.2, G101*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.5</v>
       </c>
       <c r="I101" t="s">
@@ -8036,11 +8183,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G102" s="5">
-        <f>F102-E102</f>
+        <f t="shared" si="6"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H102" s="3">
-        <f>IF(F102&gt;50, G102*0.2, G102*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I102" t="s">
@@ -8073,11 +8220,11 @@
         <v>124</v>
       </c>
       <c r="G103" s="5">
-        <f>F103-E103</f>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="H103" s="3">
-        <f>IF(F103&gt;50, G103*0.2, G103*0.1)</f>
+        <f t="shared" si="7"/>
         <v>12.8</v>
       </c>
       <c r="I103" t="s">
@@ -8110,11 +8257,11 @@
         <v>16.3</v>
       </c>
       <c r="G104" s="5">
-        <f>F104-E104</f>
+        <f t="shared" si="6"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H104" s="3">
-        <f>IF(F104&gt;50, G104*0.2, G104*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I104" t="s">
@@ -8147,11 +8294,11 @@
         <v>16.3</v>
       </c>
       <c r="G105" s="5">
-        <f>F105-E105</f>
+        <f t="shared" si="6"/>
         <v>4.9000000000000004</v>
       </c>
       <c r="H105" s="3">
-        <f>IF(F105&gt;50, G105*0.2, G105*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.49000000000000005</v>
       </c>
       <c r="I105" t="s">
@@ -8184,11 +8331,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G106" s="5">
-        <f>F106-E106</f>
+        <f t="shared" si="6"/>
         <v>2.9999999999999991</v>
       </c>
       <c r="H106" s="3">
-        <f>IF(F106&gt;50, G106*0.2, G106*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="I106" t="s">
@@ -8221,11 +8368,11 @@
         <v>98.4</v>
       </c>
       <c r="G107" s="5">
-        <f>F107-E107</f>
+        <f t="shared" si="6"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H107" s="3">
-        <f>IF(F107&gt;50, G107*0.2, G107*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I107" t="s">
@@ -8258,11 +8405,11 @@
         <v>8</v>
       </c>
       <c r="G108" s="5">
-        <f>F108-E108</f>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="H108" s="3">
-        <f>IF(F108&gt;50, G108*0.2, G108*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.5</v>
       </c>
       <c r="I108" t="s">
@@ -8295,11 +8442,11 @@
         <v>98.4</v>
       </c>
       <c r="G109" s="5">
-        <f>F109-E109</f>
+        <f t="shared" si="6"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H109" s="3">
-        <f>IF(F109&gt;50, G109*0.2, G109*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I109" t="s">
@@ -8332,11 +8479,11 @@
         <v>502</v>
       </c>
       <c r="G110" s="5">
-        <f>F110-E110</f>
+        <f t="shared" si="6"/>
         <v>158</v>
       </c>
       <c r="H110" s="3">
-        <f>IF(F110&gt;50, G110*0.2, G110*0.1)</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I110" t="s">
@@ -8369,11 +8516,11 @@
         <v>502</v>
       </c>
       <c r="G111" s="5">
-        <f>F111-E111</f>
+        <f t="shared" si="6"/>
         <v>158</v>
       </c>
       <c r="H111" s="3">
-        <f>IF(F111&gt;50, G111*0.2, G111*0.1)</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I111" t="s">
@@ -8406,11 +8553,11 @@
         <v>77</v>
       </c>
       <c r="G112" s="5">
-        <f>F112-E112</f>
+        <f t="shared" si="6"/>
         <v>35</v>
       </c>
       <c r="H112" s="3">
-        <f>IF(F112&gt;50, G112*0.2, G112*0.1)</f>
+        <f t="shared" si="7"/>
         <v>7</v>
       </c>
       <c r="I112" t="s">
@@ -8443,11 +8590,11 @@
         <v>77</v>
       </c>
       <c r="G113" s="5">
-        <f>F113-E113</f>
+        <f t="shared" si="6"/>
         <v>35</v>
       </c>
       <c r="H113" s="3">
-        <f>IF(F113&gt;50, G113*0.2, G113*0.1)</f>
+        <f t="shared" si="7"/>
         <v>7</v>
       </c>
       <c r="I113" t="s">
@@ -8480,11 +8627,11 @@
         <v>98.4</v>
       </c>
       <c r="G114" s="5">
-        <f>F114-E114</f>
+        <f t="shared" si="6"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H114" s="3">
-        <f>IF(F114&gt;50, G114*0.2, G114*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I114" t="s">
@@ -8517,11 +8664,11 @@
         <v>124</v>
       </c>
       <c r="G115" s="5">
-        <f>F115-E115</f>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="H115" s="3">
-        <f>IF(F115&gt;50, G115*0.2, G115*0.1)</f>
+        <f t="shared" si="7"/>
         <v>12.8</v>
       </c>
       <c r="I115" t="s">
@@ -8554,11 +8701,11 @@
         <v>502</v>
       </c>
       <c r="G116" s="5">
-        <f>F116-E116</f>
+        <f t="shared" si="6"/>
         <v>158</v>
       </c>
       <c r="H116" s="3">
-        <f>IF(F116&gt;50, G116*0.2, G116*0.1)</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I116" t="s">
@@ -8591,11 +8738,11 @@
         <v>77</v>
       </c>
       <c r="G117" s="5">
-        <f>F117-E117</f>
+        <f t="shared" si="6"/>
         <v>35</v>
       </c>
       <c r="H117" s="3">
-        <f>IF(F117&gt;50, G117*0.2, G117*0.1)</f>
+        <f t="shared" si="7"/>
         <v>7</v>
       </c>
       <c r="I117" t="s">
@@ -8628,11 +8775,11 @@
         <v>502</v>
       </c>
       <c r="G118" s="5">
-        <f>F118-E118</f>
+        <f t="shared" si="6"/>
         <v>158</v>
       </c>
       <c r="H118" s="3">
-        <f>IF(F118&gt;50, G118*0.2, G118*0.1)</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I118" t="s">
@@ -8665,11 +8812,11 @@
         <v>98.4</v>
       </c>
       <c r="G119" s="5">
-        <f>F119-E119</f>
+        <f t="shared" si="6"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H119" s="3">
-        <f>IF(F119&gt;50, G119*0.2, G119*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I119" t="s">
@@ -8702,11 +8849,11 @@
         <v>124</v>
       </c>
       <c r="G120" s="5">
-        <f>F120-E120</f>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="H120" s="3">
-        <f>IF(F120&gt;50, G120*0.2, G120*0.1)</f>
+        <f t="shared" si="7"/>
         <v>12.8</v>
       </c>
       <c r="I120" t="s">
@@ -8739,11 +8886,11 @@
         <v>124</v>
       </c>
       <c r="G121" s="5">
-        <f>F121-E121</f>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="H121" s="3">
-        <f>IF(F121&gt;50, G121*0.2, G121*0.1)</f>
+        <f t="shared" si="7"/>
         <v>12.8</v>
       </c>
       <c r="I121" t="s">
@@ -8776,11 +8923,11 @@
         <v>87</v>
       </c>
       <c r="G122" s="5">
-        <f>F122-E122</f>
+        <f t="shared" si="6"/>
         <v>42</v>
       </c>
       <c r="H122" s="3">
-        <f>IF(F122&gt;50, G122*0.2, G122*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.4</v>
       </c>
       <c r="I122" t="s">
@@ -8813,11 +8960,11 @@
         <v>502</v>
       </c>
       <c r="G123" s="5">
-        <f>F123-E123</f>
+        <f t="shared" si="6"/>
         <v>158</v>
       </c>
       <c r="H123" s="3">
-        <f>IF(F123&gt;50, G123*0.2, G123*0.1)</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I123" t="s">
@@ -8850,11 +8997,11 @@
         <v>98.4</v>
       </c>
       <c r="G124" s="5">
-        <f>F124-E124</f>
+        <f t="shared" si="6"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H124" s="3">
-        <f>IF(F124&gt;50, G124*0.2, G124*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I124" t="s">
@@ -8887,11 +9034,11 @@
         <v>87</v>
       </c>
       <c r="G125" s="5">
-        <f>F125-E125</f>
+        <f t="shared" si="6"/>
         <v>42</v>
       </c>
       <c r="H125" s="3">
-        <f>IF(F125&gt;50, G125*0.2, G125*0.1)</f>
+        <f t="shared" si="7"/>
         <v>8.4</v>
       </c>
       <c r="I125" t="s">
@@ -8924,11 +9071,11 @@
         <v>124</v>
       </c>
       <c r="G126" s="5">
-        <f>F126-E126</f>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="H126" s="3">
-        <f>IF(F126&gt;50, G126*0.2, G126*0.1)</f>
+        <f t="shared" si="7"/>
         <v>12.8</v>
       </c>
       <c r="I126" t="s">
@@ -8961,11 +9108,11 @@
         <v>7</v>
       </c>
       <c r="G127" s="5">
-        <f>F127-E127</f>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="H127" s="3">
-        <f>IF(F127&gt;50, G127*0.2, G127*0.1)</f>
+        <f t="shared" si="7"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I127" t="s">
@@ -8998,11 +9145,11 @@
         <v>502</v>
       </c>
       <c r="G128" s="5">
-        <f>F128-E128</f>
+        <f t="shared" si="6"/>
         <v>158</v>
       </c>
       <c r="H128" s="3">
-        <f>IF(F128&gt;50, G128*0.2, G128*0.1)</f>
+        <f t="shared" si="7"/>
         <v>31.6</v>
       </c>
       <c r="I128" t="s">
@@ -9035,11 +9182,11 @@
         <v>77</v>
       </c>
       <c r="G129" s="5">
-        <f>F129-E129</f>
+        <f t="shared" si="6"/>
         <v>35</v>
       </c>
       <c r="H129" s="3">
-        <f>IF(F129&gt;50, G129*0.2, G129*0.1)</f>
+        <f t="shared" si="7"/>
         <v>7</v>
       </c>
       <c r="I129" t="s">
@@ -9072,11 +9219,11 @@
         <v>98.4</v>
       </c>
       <c r="G130" s="5">
-        <f>F130-E130</f>
+        <f t="shared" ref="G130:G161" si="8">F130-E130</f>
         <v>40.100000000000009</v>
       </c>
       <c r="H130" s="3">
-        <f>IF(F130&gt;50, G130*0.2, G130*0.1)</f>
+        <f t="shared" ref="H130:H161" si="9">IF(F130&gt;50, G130*0.2, G130*0.1)</f>
         <v>8.0200000000000014</v>
       </c>
       <c r="I130" t="s">
@@ -9109,11 +9256,11 @@
         <v>87</v>
       </c>
       <c r="G131" s="5">
-        <f>F131-E131</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="H131" s="3">
-        <f>IF(F131&gt;50, G131*0.2, G131*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.4</v>
       </c>
       <c r="I131" t="s">
@@ -9146,11 +9293,11 @@
         <v>7</v>
       </c>
       <c r="G132" s="5">
-        <f>F132-E132</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="H132" s="3">
-        <f>IF(F132&gt;50, G132*0.2, G132*0.1)</f>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I132" t="s">
@@ -9183,11 +9330,11 @@
         <v>7</v>
       </c>
       <c r="G133" s="5">
-        <f>F133-E133</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="H133" s="3">
-        <f>IF(F133&gt;50, G133*0.2, G133*0.1)</f>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I133" t="s">
@@ -9220,11 +9367,11 @@
         <v>98.4</v>
       </c>
       <c r="G134" s="5">
-        <f>F134-E134</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H134" s="3">
-        <f>IF(F134&gt;50, G134*0.2, G134*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I134" t="s">
@@ -9257,11 +9404,11 @@
         <v>98.4</v>
       </c>
       <c r="G135" s="5">
-        <f>F135-E135</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H135" s="3">
-        <f>IF(F135&gt;50, G135*0.2, G135*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I135" t="s">
@@ -9294,11 +9441,11 @@
         <v>502</v>
       </c>
       <c r="G136" s="5">
-        <f>F136-E136</f>
+        <f t="shared" si="8"/>
         <v>158</v>
       </c>
       <c r="H136" s="3">
-        <f>IF(F136&gt;50, G136*0.2, G136*0.1)</f>
+        <f t="shared" si="9"/>
         <v>31.6</v>
       </c>
       <c r="I136" t="s">
@@ -9331,11 +9478,11 @@
         <v>124</v>
       </c>
       <c r="G137" s="5">
-        <f>F137-E137</f>
+        <f t="shared" si="8"/>
         <v>64</v>
       </c>
       <c r="H137" s="3">
-        <f>IF(F137&gt;50, G137*0.2, G137*0.1)</f>
+        <f t="shared" si="9"/>
         <v>12.8</v>
       </c>
       <c r="I137" t="s">
@@ -9368,11 +9515,11 @@
         <v>98.4</v>
       </c>
       <c r="G138" s="5">
-        <f>F138-E138</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H138" s="3">
-        <f>IF(F138&gt;50, G138*0.2, G138*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I138" t="s">
@@ -9405,11 +9552,11 @@
         <v>502</v>
       </c>
       <c r="G139" s="5">
-        <f>F139-E139</f>
+        <f t="shared" si="8"/>
         <v>158</v>
       </c>
       <c r="H139" s="3">
-        <f>IF(F139&gt;50, G139*0.2, G139*0.1)</f>
+        <f t="shared" si="9"/>
         <v>31.6</v>
       </c>
       <c r="I139" t="s">
@@ -9442,11 +9589,11 @@
         <v>87</v>
       </c>
       <c r="G140" s="5">
-        <f>F140-E140</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="H140" s="3">
-        <f>IF(F140&gt;50, G140*0.2, G140*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.4</v>
       </c>
       <c r="I140" t="s">
@@ -9479,11 +9626,11 @@
         <v>87</v>
       </c>
       <c r="G141" s="5">
-        <f>F141-E141</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="H141" s="3">
-        <f>IF(F141&gt;50, G141*0.2, G141*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.4</v>
       </c>
       <c r="I141" t="s">
@@ -9516,11 +9663,11 @@
         <v>7</v>
       </c>
       <c r="G142" s="5">
-        <f>F142-E142</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="H142" s="3">
-        <f>IF(F142&gt;50, G142*0.2, G142*0.1)</f>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I142" t="s">
@@ -9553,11 +9700,11 @@
         <v>124</v>
       </c>
       <c r="G143" s="5">
-        <f>F143-E143</f>
+        <f t="shared" si="8"/>
         <v>64</v>
       </c>
       <c r="H143" s="3">
-        <f>IF(F143&gt;50, G143*0.2, G143*0.1)</f>
+        <f t="shared" si="9"/>
         <v>12.8</v>
       </c>
       <c r="I143" t="s">
@@ -9590,11 +9737,11 @@
         <v>98.4</v>
       </c>
       <c r="G144" s="5">
-        <f>F144-E144</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H144" s="3">
-        <f>IF(F144&gt;50, G144*0.2, G144*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I144" t="s">
@@ -9627,11 +9774,11 @@
         <v>124</v>
       </c>
       <c r="G145" s="5">
-        <f>F145-E145</f>
+        <f t="shared" si="8"/>
         <v>64</v>
       </c>
       <c r="H145" s="3">
-        <f>IF(F145&gt;50, G145*0.2, G145*0.1)</f>
+        <f t="shared" si="9"/>
         <v>12.8</v>
       </c>
       <c r="I145" t="s">
@@ -9664,11 +9811,11 @@
         <v>87</v>
       </c>
       <c r="G146" s="5">
-        <f>F146-E146</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="H146" s="3">
-        <f>IF(F146&gt;50, G146*0.2, G146*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.4</v>
       </c>
       <c r="I146" t="s">
@@ -9701,11 +9848,11 @@
         <v>502</v>
       </c>
       <c r="G147" s="5">
-        <f>F147-E147</f>
+        <f t="shared" si="8"/>
         <v>158</v>
       </c>
       <c r="H147" s="3">
-        <f>IF(F147&gt;50, G147*0.2, G147*0.1)</f>
+        <f t="shared" si="9"/>
         <v>31.6</v>
       </c>
       <c r="I147" t="s">
@@ -9738,11 +9885,11 @@
         <v>98.4</v>
       </c>
       <c r="G148" s="5">
-        <f>F148-E148</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H148" s="3">
-        <f>IF(F148&gt;50, G148*0.2, G148*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I148" t="s">
@@ -9775,11 +9922,11 @@
         <v>7</v>
       </c>
       <c r="G149" s="5">
-        <f>F149-E149</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="H149" s="3">
-        <f>IF(F149&gt;50, G149*0.2, G149*0.1)</f>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I149" t="s">
@@ -9812,11 +9959,11 @@
         <v>502</v>
       </c>
       <c r="G150" s="5">
-        <f>F150-E150</f>
+        <f t="shared" si="8"/>
         <v>158</v>
       </c>
       <c r="H150" s="3">
-        <f>IF(F150&gt;50, G150*0.2, G150*0.1)</f>
+        <f t="shared" si="9"/>
         <v>31.6</v>
       </c>
       <c r="I150" t="s">
@@ -9849,11 +9996,11 @@
         <v>124</v>
       </c>
       <c r="G151" s="5">
-        <f>F151-E151</f>
+        <f t="shared" si="8"/>
         <v>64</v>
       </c>
       <c r="H151" s="3">
-        <f>IF(F151&gt;50, G151*0.2, G151*0.1)</f>
+        <f t="shared" si="9"/>
         <v>12.8</v>
       </c>
       <c r="I151" t="s">
@@ -9886,11 +10033,11 @@
         <v>124</v>
       </c>
       <c r="G152" s="5">
-        <f>F152-E152</f>
+        <f t="shared" si="8"/>
         <v>64</v>
       </c>
       <c r="H152" s="3">
-        <f>IF(F152&gt;50, G152*0.2, G152*0.1)</f>
+        <f t="shared" si="9"/>
         <v>12.8</v>
       </c>
       <c r="I152" t="s">
@@ -9923,11 +10070,11 @@
         <v>87</v>
       </c>
       <c r="G153" s="5">
-        <f>F153-E153</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="H153" s="3">
-        <f>IF(F153&gt;50, G153*0.2, G153*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.4</v>
       </c>
       <c r="I153" t="s">
@@ -9960,11 +10107,11 @@
         <v>502</v>
       </c>
       <c r="G154" s="5">
-        <f>F154-E154</f>
+        <f t="shared" si="8"/>
         <v>158</v>
       </c>
       <c r="H154" s="3">
-        <f>IF(F154&gt;50, G154*0.2, G154*0.1)</f>
+        <f t="shared" si="9"/>
         <v>31.6</v>
       </c>
       <c r="I154" t="s">
@@ -9997,11 +10144,11 @@
         <v>98.4</v>
       </c>
       <c r="G155" s="5">
-        <f>F155-E155</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H155" s="3">
-        <f>IF(F155&gt;50, G155*0.2, G155*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I155" t="s">
@@ -10034,11 +10181,11 @@
         <v>87</v>
       </c>
       <c r="G156" s="5">
-        <f>F156-E156</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="H156" s="3">
-        <f>IF(F156&gt;50, G156*0.2, G156*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.4</v>
       </c>
       <c r="I156" t="s">
@@ -10071,11 +10218,11 @@
         <v>124</v>
       </c>
       <c r="G157" s="5">
-        <f>F157-E157</f>
+        <f t="shared" si="8"/>
         <v>64</v>
       </c>
       <c r="H157" s="3">
-        <f>IF(F157&gt;50, G157*0.2, G157*0.1)</f>
+        <f t="shared" si="9"/>
         <v>12.8</v>
       </c>
       <c r="I157" t="s">
@@ -10108,11 +10255,11 @@
         <v>7</v>
       </c>
       <c r="G158" s="5">
-        <f>F158-E158</f>
+        <f t="shared" si="8"/>
         <v>3</v>
       </c>
       <c r="H158" s="3">
-        <f>IF(F158&gt;50, G158*0.2, G158*0.1)</f>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I158" t="s">
@@ -10145,11 +10292,11 @@
         <v>502</v>
       </c>
       <c r="G159" s="5">
-        <f>F159-E159</f>
+        <f t="shared" si="8"/>
         <v>158</v>
       </c>
       <c r="H159" s="3">
-        <f>IF(F159&gt;50, G159*0.2, G159*0.1)</f>
+        <f t="shared" si="9"/>
         <v>31.6</v>
       </c>
       <c r="I159" t="s">
@@ -10182,11 +10329,11 @@
         <v>77</v>
       </c>
       <c r="G160" s="5">
-        <f>F160-E160</f>
+        <f t="shared" si="8"/>
         <v>35</v>
       </c>
       <c r="H160" s="3">
-        <f>IF(F160&gt;50, G160*0.2, G160*0.1)</f>
+        <f t="shared" si="9"/>
         <v>7</v>
       </c>
       <c r="I160" t="s">
@@ -10219,11 +10366,11 @@
         <v>98.4</v>
       </c>
       <c r="G161" s="5">
-        <f>F161-E161</f>
+        <f t="shared" si="8"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H161" s="3">
-        <f>IF(F161&gt;50, G161*0.2, G161*0.1)</f>
+        <f t="shared" si="9"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I161" t="s">
@@ -10256,11 +10403,11 @@
         <v>87</v>
       </c>
       <c r="G162" s="5">
-        <f>F162-E162</f>
+        <f t="shared" ref="G162:G193" si="10">F162-E162</f>
         <v>42</v>
       </c>
       <c r="H162" s="3">
-        <f>IF(F162&gt;50, G162*0.2, G162*0.1)</f>
+        <f t="shared" ref="H162:H193" si="11">IF(F162&gt;50, G162*0.2, G162*0.1)</f>
         <v>8.4</v>
       </c>
       <c r="I162" t="s">
@@ -10293,11 +10440,11 @@
         <v>7</v>
       </c>
       <c r="G163" s="5">
-        <f>F163-E163</f>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="H163" s="3">
-        <f>IF(F163&gt;50, G163*0.2, G163*0.1)</f>
+        <f t="shared" si="11"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I163" t="s">
@@ -10330,11 +10477,11 @@
         <v>7</v>
       </c>
       <c r="G164" s="5">
-        <f>F164-E164</f>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="H164" s="3">
-        <f>IF(F164&gt;50, G164*0.2, G164*0.1)</f>
+        <f t="shared" si="11"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="I164" t="s">
@@ -10367,11 +10514,11 @@
         <v>98.4</v>
       </c>
       <c r="G165" s="5">
-        <f>F165-E165</f>
+        <f t="shared" si="10"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H165" s="3">
-        <f>IF(F165&gt;50, G165*0.2, G165*0.1)</f>
+        <f t="shared" si="11"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I165" t="s">
@@ -10404,11 +10551,11 @@
         <v>98.4</v>
       </c>
       <c r="G166" s="5">
-        <f>F166-E166</f>
+        <f t="shared" si="10"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H166" s="3">
-        <f>IF(F166&gt;50, G166*0.2, G166*0.1)</f>
+        <f t="shared" si="11"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I166" t="s">
@@ -10441,11 +10588,11 @@
         <v>502</v>
       </c>
       <c r="G167" s="5">
-        <f>F167-E167</f>
+        <f t="shared" si="10"/>
         <v>158</v>
       </c>
       <c r="H167" s="3">
-        <f>IF(F167&gt;50, G167*0.2, G167*0.1)</f>
+        <f t="shared" si="11"/>
         <v>31.6</v>
       </c>
       <c r="I167" t="s">
@@ -10478,11 +10625,11 @@
         <v>124</v>
       </c>
       <c r="G168" s="5">
-        <f>F168-E168</f>
+        <f t="shared" si="10"/>
         <v>64</v>
       </c>
       <c r="H168" s="3">
-        <f>IF(F168&gt;50, G168*0.2, G168*0.1)</f>
+        <f t="shared" si="11"/>
         <v>12.8</v>
       </c>
       <c r="I168" t="s">
@@ -10515,11 +10662,11 @@
         <v>98.4</v>
       </c>
       <c r="G169" s="5">
-        <f>F169-E169</f>
+        <f t="shared" si="10"/>
         <v>40.100000000000009</v>
       </c>
       <c r="H169" s="3">
-        <f>IF(F169&gt;50, G169*0.2, G169*0.1)</f>
+        <f t="shared" si="11"/>
         <v>8.0200000000000014</v>
       </c>
       <c r="I169" t="s">
@@ -10552,11 +10699,11 @@
         <v>502</v>
       </c>
       <c r="G170" s="5">
-        <f>F170-E170</f>
+        <f t="shared" si="10"/>
         <v>158</v>
       </c>
       <c r="H170" s="3">
-        <f>IF(F170&gt;50, G170*0.2, G170*0.1)</f>
+        <f t="shared" si="11"/>
         <v>31.6</v>
       </c>
       <c r="I170" t="s">
@@ -10589,11 +10736,11 @@
         <v>87</v>
       </c>
       <c r="G171" s="5">
-        <f>F171-E171</f>
+        <f t="shared" si="10"/>
         <v>42</v>
       </c>
       <c r="H171" s="3">
-        <f>IF(F171&gt;50, G171*0.2, G171*0.1)</f>
+        <f t="shared" si="11"/>
         <v>8.4</v>
       </c>
       <c r="I171" t="s">
@@ -10626,11 +10773,11 @@
         <v>87</v>
       </c>
       <c r="G172" s="5">
-        <f>F172-E172</f>
+        <f t="shared" si="10"/>
         <v>42</v>
       </c>
       <c r="H172" s="3">
-        <f>IF(F172&gt;50, G172*0.2, G172*0.1)</f>
+        <f t="shared" si="11"/>
         <v>8.4</v>
       </c>
       <c r="I172" t="s">
@@ -10643,17 +10790,18 @@
         <v>17</v>
       </c>
     </row>
-    <row r="174" spans="1:11">
-      <c r="A174" t="s">
+    <row r="174" spans="1:11" ht="31.2">
+      <c r="A174" s="10" t="s">
         <v>47</v>
       </c>
+      <c r="B174" s="10"/>
       <c r="F174" s="5">
         <f>SUM(F2:F172)</f>
         <v>17110.599999999995</v>
       </c>
     </row>
-    <row r="175" spans="1:11">
-      <c r="A175" t="s">
+    <row r="175" spans="1:11" ht="46.8">
+      <c r="A175" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F175" s="3">
@@ -10661,8 +10809,8 @@
         <v>16088.399999999994</v>
       </c>
     </row>
-    <row r="176" spans="1:11">
-      <c r="A176" t="s">
+    <row r="176" spans="1:11" ht="46.8">
+      <c r="A176" s="10" t="s">
         <v>49</v>
       </c>
       <c r="F176" s="3">

</xml_diff>